<commit_message>
Fix locale-specific artifacts in de-DE templates
</commit_message>
<xml_diff>
--- a/new/de-DE/new.xlsx
+++ b/new/de-DE/new.xlsx
@@ -20,13 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -54,7 +53,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>